<commit_message>
Collector circuits order fixed
</commit_message>
<xml_diff>
--- a/collector/Registros_Modbus.xlsx
+++ b/collector/Registros_Modbus.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="3"/>
+    <workbookView windowWidth="21600" windowHeight="9600" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ConexionDB" sheetId="4" r:id="rId1"/>
@@ -116,58 +116,58 @@
     <t>TP_Sistema PBM</t>
   </si>
   <si>
+    <t>TP_Planta de Biogas</t>
+  </si>
+  <si>
+    <t>TP_Banco de trabajo turbinas</t>
+  </si>
+  <si>
+    <t>TP_Tunel de viento - Potencia</t>
+  </si>
+  <si>
     <t>TP_Analizador Biogas</t>
   </si>
   <si>
-    <t>TP_Planta de Biogas</t>
-  </si>
-  <si>
-    <t>TP_Tunel de viento - Potencia</t>
-  </si>
-  <si>
     <t>TP_Ventilador sistema eolico</t>
   </si>
   <si>
     <t>TP_Torre de enfriamiento</t>
   </si>
   <si>
-    <t>TP_Banco de trabajo turbinas</t>
-  </si>
-  <si>
     <t>TP_Tablero Paneles</t>
   </si>
   <si>
+    <t>TP_Tunel de viento - control</t>
+  </si>
+  <si>
+    <t>TP_Modulo control turbinas</t>
+  </si>
+  <si>
+    <t>TP_Modulo fotovoltaico eolico</t>
+  </si>
+  <si>
+    <t>TP_Iluminacion Smartgrid</t>
+  </si>
+  <si>
+    <t>TP_Nevera Biogas</t>
+  </si>
+  <si>
+    <t>TP_Meson Sala Biogas</t>
+  </si>
+  <si>
+    <t>TP_Mesa Biogas Fotovoltaico</t>
+  </si>
+  <si>
+    <t>TP_Iluminacion fotovoltaico</t>
+  </si>
+  <si>
     <t>TP_Iluminacion Biogas</t>
   </si>
   <si>
     <t>TP_Video Wall Smart Grid</t>
   </si>
   <si>
-    <t>TP_Iluminacion fotovoltaico</t>
-  </si>
-  <si>
     <t>TP_Video Controller Smart Grid</t>
-  </si>
-  <si>
-    <t>TP_Iluminacion Smartgrid</t>
-  </si>
-  <si>
-    <t>TP_Mesa Biogas Fotovoltaico</t>
-  </si>
-  <si>
-    <t>TP_Nevera Biogas</t>
-  </si>
-  <si>
-    <t>TP_Meson Sala Biogas</t>
-  </si>
-  <si>
-    <t>TP_Tunel de viento - control</t>
-  </si>
-  <si>
-    <t>TP_Modulo fotovoltaico eolico</t>
-  </si>
-  <si>
-    <t>TP_Modulo control turbinas</t>
   </si>
   <si>
     <t>Address Hex</t>
@@ -3322,8 +3322,8 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C118"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="2"/>
+  <dimension ref="A1:E118"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
@@ -3355,7 +3355,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3365,8 +3365,10 @@
       <c r="C3" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="D3" s="1"/>
+      <c r="E3" s="13"/>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3376,8 +3378,10 @@
       <c r="C4" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="D4"/>
+      <c r="E4" s="13"/>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3387,8 +3391,10 @@
       <c r="C5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="D5"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3398,8 +3404,10 @@
       <c r="C6" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="D6"/>
+      <c r="E6" s="13"/>
+    </row>
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3409,8 +3417,10 @@
       <c r="C7" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="D7"/>
+      <c r="E7" s="13"/>
+    </row>
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3420,8 +3430,10 @@
       <c r="C8" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="D8"/>
+      <c r="E8" s="13"/>
+    </row>
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3431,8 +3443,10 @@
       <c r="C9" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="D9"/>
+      <c r="E9" s="13"/>
+    </row>
+    <row r="10" spans="1:5">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3442,8 +3456,10 @@
       <c r="C10" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="D10"/>
+      <c r="E10" s="13"/>
+    </row>
+    <row r="11" spans="1:5">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3453,8 +3469,10 @@
       <c r="C11" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="D11"/>
+      <c r="E11" s="13"/>
+    </row>
+    <row r="12" spans="1:5">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3464,8 +3482,10 @@
       <c r="C12" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="D12"/>
+      <c r="E12" s="13"/>
+    </row>
+    <row r="13" spans="1:5">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3475,8 +3495,10 @@
       <c r="C13" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="D13"/>
+      <c r="E13" s="13"/>
+    </row>
+    <row r="14" spans="1:5">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3486,8 +3508,10 @@
       <c r="C14" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="D14"/>
+      <c r="E14" s="13"/>
+    </row>
+    <row r="15" spans="1:5">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3497,8 +3521,10 @@
       <c r="C15" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="D15"/>
+      <c r="E15" s="13"/>
+    </row>
+    <row r="16" spans="1:5">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3508,8 +3534,10 @@
       <c r="C16" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="17" spans="1:3">
+      <c r="D16"/>
+      <c r="E16" s="13"/>
+    </row>
+    <row r="17" spans="1:5">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3519,8 +3547,10 @@
       <c r="C17" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="18" spans="1:3">
+      <c r="D17"/>
+      <c r="E17" s="13"/>
+    </row>
+    <row r="18" spans="1:5">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3530,8 +3560,10 @@
       <c r="C18" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="19" spans="1:3">
+      <c r="D18"/>
+      <c r="E18" s="13"/>
+    </row>
+    <row r="19" spans="1:5">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3541,8 +3573,10 @@
       <c r="C19" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="20" spans="1:3">
+      <c r="D19"/>
+      <c r="E19" s="13"/>
+    </row>
+    <row r="20" spans="1:5">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3552,8 +3586,10 @@
       <c r="C20" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="21" spans="1:3">
+      <c r="D20"/>
+      <c r="E20" s="13"/>
+    </row>
+    <row r="21" spans="1:5">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3563,6 +3599,8 @@
       <c r="C21" t="s">
         <v>11</v>
       </c>
+      <c r="D21"/>
+      <c r="E21" s="13"/>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="14"/>

</xml_diff>